<commit_message>
Remove the duplicate Calvin Klein and Murine listings; draft bundle SKU codes
Done on the store on 25 Sep 2026, logged in setup/product-import/dedupe-2026-09-25/
with the full before state of all four products:

- Calvin Klein Eternity For Men (created 23 Sep by the Anas-product-image-upload
  app, POS only) deleted after its 1080px image replaced Ck Men's 600px copy of
  the same picture.
- Murine: kept the 10Ml listing (valid barcode, real photo), gave it the box's
  "Relief" wording, deleted the other, redirected its URL.

The barcode check list drops the two deleted products (74 -> 72 rows).
bundle-sku-draft-2026-09-25.csv holds text SKUs for the 8 bundles with invented
numbers; not applied until Keelan confirms whether the till matches on SKU.

Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/setup/product-import/barcode-check-2026-09-25.xlsx
+++ b/setup/product-import/barcode-check-2026-09-25.xlsx
@@ -10,7 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Check against the box" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Check against the box'!$A$1:$J$75</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Check against the box'!$A$1:$J$73</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -426,7 +426,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J75"/>
+  <dimension ref="A1:J73"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -792,29 +792,21 @@
           <t>Leading zero lost</t>
         </is>
       </c>
-      <c r="C9" s="2" t="inlineStr">
-        <is>
-          <t>COLLISION: already the barcode of Ck Men 50Ml Edt Spr</t>
-        </is>
-      </c>
+      <c r="C9" s="2" t="inlineStr"/>
       <c r="D9" s="2" t="inlineStr">
         <is>
-          <t>Calvin Klein Eternity For Men 50Ml Edt Spr</t>
+          <t>Lil Critters Immune C (60 Pk)</t>
         </is>
       </c>
       <c r="E9" s="2" t="inlineStr">
         <is>
-          <t>31655644295</t>
-        </is>
-      </c>
-      <c r="F9" s="2" t="inlineStr">
-        <is>
-          <t>31655644295</t>
-        </is>
-      </c>
+          <t>27917017594</t>
+        </is>
+      </c>
+      <c r="F9" s="2" t="inlineStr"/>
       <c r="G9" s="2" t="inlineStr">
         <is>
-          <t>031655644295</t>
+          <t>027917017594</t>
         </is>
       </c>
       <c r="H9" s="3" t="inlineStr"/>
@@ -825,7 +817,7 @@
       </c>
       <c r="J9" s="2" t="inlineStr">
         <is>
-          <t>https://admin.shopify.com/store/mccormackpharmacy/products/16024784666955</t>
+          <t>https://admin.shopify.com/store/mccormackpharmacy/products/15671394500939</t>
         </is>
       </c>
     </row>
@@ -841,18 +833,18 @@
       <c r="C10" s="2" t="inlineStr"/>
       <c r="D10" s="2" t="inlineStr">
         <is>
-          <t>Lil Critters Immune C (60 Pk)</t>
+          <t>Marc Jacobs Daisy 100Ml Edt</t>
         </is>
       </c>
       <c r="E10" s="2" t="inlineStr">
         <is>
-          <t>27917017594</t>
+          <t>31655513034</t>
         </is>
       </c>
       <c r="F10" s="2" t="inlineStr"/>
       <c r="G10" s="2" t="inlineStr">
         <is>
-          <t>027917017594</t>
+          <t>031655513034</t>
         </is>
       </c>
       <c r="H10" s="3" t="inlineStr"/>
@@ -863,7 +855,7 @@
       </c>
       <c r="J10" s="2" t="inlineStr">
         <is>
-          <t>https://admin.shopify.com/store/mccormackpharmacy/products/15671394500939</t>
+          <t>https://admin.shopify.com/store/mccormackpharmacy/products/15671398695243</t>
         </is>
       </c>
     </row>
@@ -879,18 +871,22 @@
       <c r="C11" s="2" t="inlineStr"/>
       <c r="D11" s="2" t="inlineStr">
         <is>
-          <t>Marc Jacobs Daisy 100Ml Edt</t>
+          <t>Solgar 7 Joint Support 30 Caps</t>
         </is>
       </c>
       <c r="E11" s="2" t="inlineStr">
         <is>
-          <t>31655513034</t>
-        </is>
-      </c>
-      <c r="F11" s="2" t="inlineStr"/>
+          <t>33984504974</t>
+        </is>
+      </c>
+      <c r="F11" s="2" t="inlineStr">
+        <is>
+          <t>33984504974</t>
+        </is>
+      </c>
       <c r="G11" s="2" t="inlineStr">
         <is>
-          <t>031655513034</t>
+          <t>033984504974</t>
         </is>
       </c>
       <c r="H11" s="3" t="inlineStr"/>
@@ -901,7 +897,7 @@
       </c>
       <c r="J11" s="2" t="inlineStr">
         <is>
-          <t>https://admin.shopify.com/store/mccormackpharmacy/products/15671398695243</t>
+          <t>https://admin.shopify.com/store/mccormackpharmacy/products/16024784109899</t>
         </is>
       </c>
     </row>
@@ -917,22 +913,22 @@
       <c r="C12" s="2" t="inlineStr"/>
       <c r="D12" s="2" t="inlineStr">
         <is>
-          <t>Solgar 7 Joint Support 30 Caps</t>
+          <t>Solgar Magnesium L-Threonate 60 Capsules</t>
         </is>
       </c>
       <c r="E12" s="2" t="inlineStr">
         <is>
-          <t>33984504974</t>
+          <t>33984015777</t>
         </is>
       </c>
       <c r="F12" s="2" t="inlineStr">
         <is>
-          <t>33984504974</t>
+          <t>33984015777</t>
         </is>
       </c>
       <c r="G12" s="2" t="inlineStr">
         <is>
-          <t>033984504974</t>
+          <t>033984015777</t>
         </is>
       </c>
       <c r="H12" s="3" t="inlineStr"/>
@@ -943,49 +939,45 @@
       </c>
       <c r="J12" s="2" t="inlineStr">
         <is>
-          <t>https://admin.shopify.com/store/mccormackpharmacy/products/16024784109899</t>
+          <t>https://admin.shopify.com/store/mccormackpharmacy/products/16024784535883</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="B13" s="2" t="inlineStr">
         <is>
-          <t>Leading zero lost</t>
+          <t>Extra or padded digits</t>
         </is>
       </c>
       <c r="C13" s="2" t="inlineStr"/>
       <c r="D13" s="2" t="inlineStr">
         <is>
-          <t>Solgar Magnesium L-Threonate 60 Capsules</t>
+          <t>2 Piece Ladies Set Adoor</t>
         </is>
       </c>
       <c r="E13" s="2" t="inlineStr">
         <is>
-          <t>33984015777</t>
-        </is>
-      </c>
-      <c r="F13" s="2" t="inlineStr">
-        <is>
-          <t>33984015777</t>
-        </is>
-      </c>
+          <t>6294015186407</t>
+        </is>
+      </c>
+      <c r="F13" s="2" t="inlineStr"/>
       <c r="G13" s="2" t="inlineStr">
         <is>
-          <t>033984015777</t>
+          <t>629401518640</t>
         </is>
       </c>
       <c r="H13" s="3" t="inlineStr"/>
       <c r="I13" s="2" t="inlineStr">
         <is>
-          <t>Looks like Excel dropped the leading 0. Check the box shows the suggested number.</t>
+          <t>Too many digits; trimming gives a number that passes the check, but 1 in 10 wrong numbers also pass. Check the box.</t>
         </is>
       </c>
       <c r="J13" s="2" t="inlineStr">
         <is>
-          <t>https://admin.shopify.com/store/mccormackpharmacy/products/16024784535883</t>
+          <t>https://admin.shopify.com/store/mccormackpharmacy/products/15671338926411</t>
         </is>
       </c>
     </row>
@@ -1001,18 +993,18 @@
       <c r="C14" s="2" t="inlineStr"/>
       <c r="D14" s="2" t="inlineStr">
         <is>
-          <t>2 Piece Ladies Set Adoor</t>
+          <t>Caldesene Medicated Powder 100G</t>
         </is>
       </c>
       <c r="E14" s="2" t="inlineStr">
         <is>
-          <t>6294015186407</t>
+          <t>50995627273520</t>
         </is>
       </c>
       <c r="F14" s="2" t="inlineStr"/>
       <c r="G14" s="2" t="inlineStr">
         <is>
-          <t>629401518640</t>
+          <t>5099562727352</t>
         </is>
       </c>
       <c r="H14" s="3" t="inlineStr"/>
@@ -1023,7 +1015,7 @@
       </c>
       <c r="J14" s="2" t="inlineStr">
         <is>
-          <t>https://admin.shopify.com/store/mccormackpharmacy/products/15671338926411</t>
+          <t>https://admin.shopify.com/store/mccormackpharmacy/products/15671284498763</t>
         </is>
       </c>
     </row>
@@ -1039,18 +1031,18 @@
       <c r="C15" s="2" t="inlineStr"/>
       <c r="D15" s="2" t="inlineStr">
         <is>
-          <t>Caldesene Medicated Powder 100G</t>
+          <t>Ck Eternity Mens 50Ml Edt Spr</t>
         </is>
       </c>
       <c r="E15" s="2" t="inlineStr">
         <is>
-          <t>50995627273520</t>
+          <t>0883001053040</t>
         </is>
       </c>
       <c r="F15" s="2" t="inlineStr"/>
       <c r="G15" s="2" t="inlineStr">
         <is>
-          <t>5099562727352</t>
+          <t>088300105304</t>
         </is>
       </c>
       <c r="H15" s="3" t="inlineStr"/>
@@ -1061,7 +1053,7 @@
       </c>
       <c r="J15" s="2" t="inlineStr">
         <is>
-          <t>https://admin.shopify.com/store/mccormackpharmacy/products/15671284498763</t>
+          <t>https://admin.shopify.com/store/mccormackpharmacy/products/15671321952587</t>
         </is>
       </c>
     </row>
@@ -1077,18 +1069,18 @@
       <c r="C16" s="2" t="inlineStr"/>
       <c r="D16" s="2" t="inlineStr">
         <is>
-          <t>Ck Eternity Mens 50Ml Edt Spr</t>
+          <t>Eucerin 10% Urea Foot Cream</t>
         </is>
       </c>
       <c r="E16" s="2" t="inlineStr">
         <is>
-          <t>0883001053040</t>
+          <t>40058000361011</t>
         </is>
       </c>
       <c r="F16" s="2" t="inlineStr"/>
       <c r="G16" s="2" t="inlineStr">
         <is>
-          <t>088300105304</t>
+          <t>4005800036101</t>
         </is>
       </c>
       <c r="H16" s="3" t="inlineStr"/>
@@ -1099,7 +1091,7 @@
       </c>
       <c r="J16" s="2" t="inlineStr">
         <is>
-          <t>https://admin.shopify.com/store/mccormackpharmacy/products/15671321952587</t>
+          <t>https://admin.shopify.com/store/mccormackpharmacy/products/15671409246539</t>
         </is>
       </c>
     </row>
@@ -1115,18 +1107,18 @@
       <c r="C17" s="2" t="inlineStr"/>
       <c r="D17" s="2" t="inlineStr">
         <is>
-          <t>Eucerin 10% Urea Foot Cream</t>
+          <t>Hugo Extreme Mens 75Ml Edp Spr</t>
         </is>
       </c>
       <c r="E17" s="2" t="inlineStr">
         <is>
-          <t>40058000361011</t>
+          <t>36163016223380</t>
         </is>
       </c>
       <c r="F17" s="2" t="inlineStr"/>
       <c r="G17" s="2" t="inlineStr">
         <is>
-          <t>4005800036101</t>
+          <t>3616301622338</t>
         </is>
       </c>
       <c r="H17" s="3" t="inlineStr"/>
@@ -1137,7 +1129,7 @@
       </c>
       <c r="J17" s="2" t="inlineStr">
         <is>
-          <t>https://admin.shopify.com/store/mccormackpharmacy/products/15671409246539</t>
+          <t>https://admin.shopify.com/store/mccormackpharmacy/products/15671349805387</t>
         </is>
       </c>
     </row>
@@ -1153,18 +1145,18 @@
       <c r="C18" s="2" t="inlineStr"/>
       <c r="D18" s="2" t="inlineStr">
         <is>
-          <t>Hugo Extreme Mens 75Ml Edp Spr</t>
+          <t>Mam Air 12+ Months (White/Blue Fox)</t>
         </is>
       </c>
       <c r="E18" s="2" t="inlineStr">
         <is>
-          <t>36163016223380</t>
+          <t>900161671022300</t>
         </is>
       </c>
       <c r="F18" s="2" t="inlineStr"/>
       <c r="G18" s="2" t="inlineStr">
         <is>
-          <t>3616301622338</t>
+          <t>9001616710223</t>
         </is>
       </c>
       <c r="H18" s="3" t="inlineStr"/>
@@ -1175,7 +1167,7 @@
       </c>
       <c r="J18" s="2" t="inlineStr">
         <is>
-          <t>https://admin.shopify.com/store/mccormackpharmacy/products/15671349805387</t>
+          <t>https://admin.shopify.com/store/mccormackpharmacy/products/15671319003467</t>
         </is>
       </c>
     </row>
@@ -1188,21 +1180,25 @@
           <t>Extra or padded digits</t>
         </is>
       </c>
-      <c r="C19" s="2" t="inlineStr"/>
+      <c r="C19" s="2" t="inlineStr">
+        <is>
+          <t>COLLISION: already the barcode of Mam Clip Double Set 0+Months Blue</t>
+        </is>
+      </c>
       <c r="D19" s="2" t="inlineStr">
         <is>
-          <t>Mam Air 12+ Months (White/Blue Fox)</t>
+          <t>Mam Clip Double Set 0+Months</t>
         </is>
       </c>
       <c r="E19" s="2" t="inlineStr">
         <is>
-          <t>900161671022300</t>
+          <t>90016162052311</t>
         </is>
       </c>
       <c r="F19" s="2" t="inlineStr"/>
       <c r="G19" s="2" t="inlineStr">
         <is>
-          <t>9001616710223</t>
+          <t>9001616205231</t>
         </is>
       </c>
       <c r="H19" s="3" t="inlineStr"/>
@@ -1213,7 +1209,7 @@
       </c>
       <c r="J19" s="2" t="inlineStr">
         <is>
-          <t>https://admin.shopify.com/store/mccormackpharmacy/products/15671319003467</t>
+          <t>https://admin.shopify.com/store/mccormackpharmacy/products/15671294099787</t>
         </is>
       </c>
     </row>
@@ -1228,23 +1224,23 @@
       </c>
       <c r="C20" s="2" t="inlineStr">
         <is>
-          <t>COLLISION: already the barcode of Mam Clip Double Set 0+Months Blue</t>
+          <t>COLLISION: already the barcode of Mam Easy Start Anti Colic 2+Months Pink</t>
         </is>
       </c>
       <c r="D20" s="2" t="inlineStr">
         <is>
-          <t>Mam Clip Double Set 0+Months</t>
+          <t>Mam Easy Start Anti Colic 2+Months Light Pink</t>
         </is>
       </c>
       <c r="E20" s="2" t="inlineStr">
         <is>
-          <t>90016162052311</t>
+          <t>90016166699341</t>
         </is>
       </c>
       <c r="F20" s="2" t="inlineStr"/>
       <c r="G20" s="2" t="inlineStr">
         <is>
-          <t>9001616205231</t>
+          <t>9001616669934</t>
         </is>
       </c>
       <c r="H20" s="3" t="inlineStr"/>
@@ -1255,7 +1251,7 @@
       </c>
       <c r="J20" s="2" t="inlineStr">
         <is>
-          <t>https://admin.shopify.com/store/mccormackpharmacy/products/15671294099787</t>
+          <t>https://admin.shopify.com/store/mccormackpharmacy/products/15671332340043</t>
         </is>
       </c>
     </row>
@@ -1270,23 +1266,23 @@
       </c>
       <c r="C21" s="2" t="inlineStr">
         <is>
-          <t>COLLISION: already the barcode of Mam Easy Start Anti Colic 2+Months Pink</t>
+          <t>COLLISION: suggested number would land on 2 products</t>
         </is>
       </c>
       <c r="D21" s="2" t="inlineStr">
         <is>
-          <t>Mam Easy Start Anti Colic 2+Months Light Pink</t>
+          <t>Mam Original 6+ Months (Blue/White)</t>
         </is>
       </c>
       <c r="E21" s="2" t="inlineStr">
         <is>
-          <t>90016166699341</t>
+          <t>90016162020180</t>
         </is>
       </c>
       <c r="F21" s="2" t="inlineStr"/>
       <c r="G21" s="2" t="inlineStr">
         <is>
-          <t>9001616669934</t>
+          <t>9001616202018</t>
         </is>
       </c>
       <c r="H21" s="3" t="inlineStr"/>
@@ -1297,7 +1293,7 @@
       </c>
       <c r="J21" s="2" t="inlineStr">
         <is>
-          <t>https://admin.shopify.com/store/mccormackpharmacy/products/15671332340043</t>
+          <t>https://admin.shopify.com/store/mccormackpharmacy/products/15671290757451</t>
         </is>
       </c>
     </row>
@@ -1317,12 +1313,12 @@
       </c>
       <c r="D22" s="2" t="inlineStr">
         <is>
-          <t>Mam Original 6+ Months (Blue/White)</t>
+          <t>Mam Original 6+ Months (Pink Cat/Blue Flowers)</t>
         </is>
       </c>
       <c r="E22" s="2" t="inlineStr">
         <is>
-          <t>90016162020180</t>
+          <t>900161620201800</t>
         </is>
       </c>
       <c r="F22" s="2" t="inlineStr"/>
@@ -1339,7 +1335,7 @@
       </c>
       <c r="J22" s="2" t="inlineStr">
         <is>
-          <t>https://admin.shopify.com/store/mccormackpharmacy/products/15671290757451</t>
+          <t>https://admin.shopify.com/store/mccormackpharmacy/products/15671392108875</t>
         </is>
       </c>
     </row>
@@ -1359,18 +1355,18 @@
       </c>
       <c r="D23" s="2" t="inlineStr">
         <is>
-          <t>Mam Original 6+ Months (Pink Cat/Blue Flowers)</t>
+          <t>Mam Original Night 0+ Months (Light Purple/Light Pink Stars)</t>
         </is>
       </c>
       <c r="E23" s="2" t="inlineStr">
         <is>
-          <t>900161620201800</t>
+          <t>900161690829300</t>
         </is>
       </c>
       <c r="F23" s="2" t="inlineStr"/>
       <c r="G23" s="2" t="inlineStr">
         <is>
-          <t>9001616202018</t>
+          <t>9001616908293</t>
         </is>
       </c>
       <c r="H23" s="3" t="inlineStr"/>
@@ -1381,7 +1377,7 @@
       </c>
       <c r="J23" s="2" t="inlineStr">
         <is>
-          <t>https://admin.shopify.com/store/mccormackpharmacy/products/15671392108875</t>
+          <t>https://admin.shopify.com/store/mccormackpharmacy/products/15671322673483</t>
         </is>
       </c>
     </row>
@@ -1401,12 +1397,12 @@
       </c>
       <c r="D24" s="2" t="inlineStr">
         <is>
-          <t>Mam Original Night 0+ Months (Light Purple/Light Pink Stars)</t>
+          <t>Mam Original Night 0+ Months (White)</t>
         </is>
       </c>
       <c r="E24" s="2" t="inlineStr">
         <is>
-          <t>900161690829300</t>
+          <t>90016169082930</t>
         </is>
       </c>
       <c r="F24" s="2" t="inlineStr"/>
@@ -1423,7 +1419,7 @@
       </c>
       <c r="J24" s="2" t="inlineStr">
         <is>
-          <t>https://admin.shopify.com/store/mccormackpharmacy/products/15671322673483</t>
+          <t>https://admin.shopify.com/store/mccormackpharmacy/products/15671361962315</t>
         </is>
       </c>
     </row>
@@ -1438,23 +1434,23 @@
       </c>
       <c r="C25" s="2" t="inlineStr">
         <is>
-          <t>COLLISION: suggested number would land on 2 products</t>
+          <t>COLLISION: suggested number would land on 2 products | COLLISION: already the barcode of Mam Night Soother 12Mths+ Silicone</t>
         </is>
       </c>
       <c r="D25" s="2" t="inlineStr">
         <is>
-          <t>Mam Original Night 0+ Months (White)</t>
+          <t>Mam Original Night 12+ Months (Navy/White)</t>
         </is>
       </c>
       <c r="E25" s="2" t="inlineStr">
         <is>
-          <t>90016169082930</t>
+          <t>90016167096540</t>
         </is>
       </c>
       <c r="F25" s="2" t="inlineStr"/>
       <c r="G25" s="2" t="inlineStr">
         <is>
-          <t>9001616908293</t>
+          <t>9001616709654</t>
         </is>
       </c>
       <c r="H25" s="3" t="inlineStr"/>
@@ -1465,7 +1461,7 @@
       </c>
       <c r="J25" s="2" t="inlineStr">
         <is>
-          <t>https://admin.shopify.com/store/mccormackpharmacy/products/15671361962315</t>
+          <t>https://admin.shopify.com/store/mccormackpharmacy/products/15671393124683</t>
         </is>
       </c>
     </row>
@@ -1485,12 +1481,12 @@
       </c>
       <c r="D26" s="2" t="inlineStr">
         <is>
-          <t>Mam Original Night 12+ Months (Navy/White)</t>
+          <t>Mam Original Night 12+ Months (Purple Owl/White)</t>
         </is>
       </c>
       <c r="E26" s="2" t="inlineStr">
         <is>
-          <t>90016167096540</t>
+          <t>9001616709654000</t>
         </is>
       </c>
       <c r="F26" s="2" t="inlineStr"/>
@@ -1507,7 +1503,7 @@
       </c>
       <c r="J26" s="2" t="inlineStr">
         <is>
-          <t>https://admin.shopify.com/store/mccormackpharmacy/products/15671393124683</t>
+          <t>https://admin.shopify.com/store/mccormackpharmacy/products/15671374053707</t>
         </is>
       </c>
     </row>
@@ -1522,23 +1518,23 @@
       </c>
       <c r="C27" s="2" t="inlineStr">
         <is>
-          <t>COLLISION: suggested number would land on 2 products | COLLISION: already the barcode of Mam Night Soother 12Mths+ Silicone</t>
+          <t>COLLISION: suggested number would land on 3 products | COLLISION: already the barcode of Mam Original Night 6+Months</t>
         </is>
       </c>
       <c r="D27" s="2" t="inlineStr">
         <is>
-          <t>Mam Original Night 12+ Months (Purple Owl/White)</t>
+          <t>Mam Original Night 6+ Months (Baby Pink/ White)</t>
         </is>
       </c>
       <c r="E27" s="2" t="inlineStr">
         <is>
-          <t>9001616709654000</t>
+          <t>90016162038620000</t>
         </is>
       </c>
       <c r="F27" s="2" t="inlineStr"/>
       <c r="G27" s="2" t="inlineStr">
         <is>
-          <t>9001616709654</t>
+          <t>9001616203862</t>
         </is>
       </c>
       <c r="H27" s="3" t="inlineStr"/>
@@ -1549,7 +1545,7 @@
       </c>
       <c r="J27" s="2" t="inlineStr">
         <is>
-          <t>https://admin.shopify.com/store/mccormackpharmacy/products/15671374053707</t>
+          <t>https://admin.shopify.com/store/mccormackpharmacy/products/15671339778379</t>
         </is>
       </c>
     </row>
@@ -1569,12 +1565,12 @@
       </c>
       <c r="D28" s="2" t="inlineStr">
         <is>
-          <t>Mam Original Night 6+ Months (Baby Pink/ White)</t>
+          <t>Mam Original Night 6+ Months (Blue/White Moon)</t>
         </is>
       </c>
       <c r="E28" s="2" t="inlineStr">
         <is>
-          <t>90016162038620000</t>
+          <t>900161620386200</t>
         </is>
       </c>
       <c r="F28" s="2" t="inlineStr"/>
@@ -1591,7 +1587,7 @@
       </c>
       <c r="J28" s="2" t="inlineStr">
         <is>
-          <t>https://admin.shopify.com/store/mccormackpharmacy/products/15671339778379</t>
+          <t>https://admin.shopify.com/store/mccormackpharmacy/products/15671337517387</t>
         </is>
       </c>
     </row>
@@ -1611,12 +1607,12 @@
       </c>
       <c r="D29" s="2" t="inlineStr">
         <is>
-          <t>Mam Original Night 6+ Months (Blue/White Moon)</t>
+          <t>Mam Original Night 6+ Months (Dark Blue/Light Blue)</t>
         </is>
       </c>
       <c r="E29" s="2" t="inlineStr">
         <is>
-          <t>900161620386200</t>
+          <t>90016162038620</t>
         </is>
       </c>
       <c r="F29" s="2" t="inlineStr"/>
@@ -1633,7 +1629,7 @@
       </c>
       <c r="J29" s="2" t="inlineStr">
         <is>
-          <t>https://admin.shopify.com/store/mccormackpharmacy/products/15671337517387</t>
+          <t>https://admin.shopify.com/store/mccormackpharmacy/products/15671284793675</t>
         </is>
       </c>
     </row>
@@ -1648,23 +1644,23 @@
       </c>
       <c r="C30" s="2" t="inlineStr">
         <is>
-          <t>COLLISION: suggested number would land on 3 products | COLLISION: already the barcode of Mam Original Night 6+Months</t>
+          <t>COLLISION: already the barcode of Mam Starter Cup Night 4+Months Green</t>
         </is>
       </c>
       <c r="D30" s="2" t="inlineStr">
         <is>
-          <t>Mam Original Night 6+ Months (Dark Blue/Light Blue)</t>
+          <t>Mam Starter Cup Night 4+Months Pink</t>
         </is>
       </c>
       <c r="E30" s="2" t="inlineStr">
         <is>
-          <t>90016162038620</t>
+          <t>90016168079477</t>
         </is>
       </c>
       <c r="F30" s="2" t="inlineStr"/>
       <c r="G30" s="2" t="inlineStr">
         <is>
-          <t>9001616203862</t>
+          <t>9001616807947</t>
         </is>
       </c>
       <c r="H30" s="3" t="inlineStr"/>
@@ -1675,7 +1671,7 @@
       </c>
       <c r="J30" s="2" t="inlineStr">
         <is>
-          <t>https://admin.shopify.com/store/mccormackpharmacy/products/15671284793675</t>
+          <t>https://admin.shopify.com/store/mccormackpharmacy/products/15671291183435</t>
         </is>
       </c>
     </row>
@@ -1690,23 +1686,23 @@
       </c>
       <c r="C31" s="2" t="inlineStr">
         <is>
-          <t>COLLISION: already the barcode of Mam Starter Cup Night 4+Months Green</t>
+          <t>BUNDLE: shop-made, should have no barcode; leave blank</t>
         </is>
       </c>
       <c r="D31" s="2" t="inlineStr">
         <is>
-          <t>Mam Starter Cup Night 4+Months Pink</t>
+          <t>Pestle &amp; Mortar Brightening Bundle</t>
         </is>
       </c>
       <c r="E31" s="2" t="inlineStr">
         <is>
-          <t>90016168079477</t>
+          <t>48564985643598</t>
         </is>
       </c>
       <c r="F31" s="2" t="inlineStr"/>
       <c r="G31" s="2" t="inlineStr">
         <is>
-          <t>9001616807947</t>
+          <t>4856498564359</t>
         </is>
       </c>
       <c r="H31" s="3" t="inlineStr"/>
@@ -1717,7 +1713,7 @@
       </c>
       <c r="J31" s="2" t="inlineStr">
         <is>
-          <t>https://admin.shopify.com/store/mccormackpharmacy/products/15671291183435</t>
+          <t>https://admin.shopify.com/store/mccormackpharmacy/products/15671259005259</t>
         </is>
       </c>
     </row>
@@ -1730,25 +1726,21 @@
           <t>Extra or padded digits</t>
         </is>
       </c>
-      <c r="C32" s="2" t="inlineStr">
-        <is>
-          <t>COLLISION: already the barcode of Murine Irritation &amp; Redness Eye Drops 10Ml</t>
-        </is>
-      </c>
+      <c r="C32" s="2" t="inlineStr"/>
       <c r="D32" s="2" t="inlineStr">
         <is>
-          <t>Murine Irritation &amp; Redness Relief Eye Drops</t>
+          <t>Revive Active Tropical 210 Sachets 7 Months Supply</t>
         </is>
       </c>
       <c r="E32" s="2" t="inlineStr">
         <is>
-          <t>50600188802040</t>
+          <t>4789625416554</t>
         </is>
       </c>
       <c r="F32" s="2" t="inlineStr"/>
       <c r="G32" s="2" t="inlineStr">
         <is>
-          <t>5060018880204</t>
+          <t>478962541655</t>
         </is>
       </c>
       <c r="H32" s="3" t="inlineStr"/>
@@ -1759,7 +1751,7 @@
       </c>
       <c r="J32" s="2" t="inlineStr">
         <is>
-          <t>https://admin.shopify.com/store/mccormackpharmacy/products/15671257596235</t>
+          <t>https://admin.shopify.com/store/mccormackpharmacy/products/15671253991755</t>
         </is>
       </c>
     </row>
@@ -1779,18 +1771,18 @@
       </c>
       <c r="D33" s="2" t="inlineStr">
         <is>
-          <t>Pestle &amp; Mortar Brightening Bundle</t>
+          <t>Unisex Festival Essentials Bundle</t>
         </is>
       </c>
       <c r="E33" s="2" t="inlineStr">
         <is>
-          <t>48564985643598</t>
+          <t>743485657575858</t>
         </is>
       </c>
       <c r="F33" s="2" t="inlineStr"/>
       <c r="G33" s="2" t="inlineStr">
         <is>
-          <t>4856498564359</t>
+          <t>7434856575758</t>
         </is>
       </c>
       <c r="H33" s="3" t="inlineStr"/>
@@ -1801,7 +1793,7 @@
       </c>
       <c r="J33" s="2" t="inlineStr">
         <is>
-          <t>https://admin.shopify.com/store/mccormackpharmacy/products/15671259005259</t>
+          <t>https://admin.shopify.com/store/mccormackpharmacy/products/15671337877835</t>
         </is>
       </c>
     </row>
@@ -1817,18 +1809,18 @@
       <c r="C34" s="2" t="inlineStr"/>
       <c r="D34" s="2" t="inlineStr">
         <is>
-          <t>Revive Active Tropical 210 Sachets 7 Months Supply</t>
+          <t>Ysl Black Opium Ladies 50Ml Edp Spr</t>
         </is>
       </c>
       <c r="E34" s="2" t="inlineStr">
         <is>
-          <t>4789625416554</t>
+          <t>33654407879190</t>
         </is>
       </c>
       <c r="F34" s="2" t="inlineStr"/>
       <c r="G34" s="2" t="inlineStr">
         <is>
-          <t>478962541655</t>
+          <t>3365440787919</t>
         </is>
       </c>
       <c r="H34" s="3" t="inlineStr"/>
@@ -1839,87 +1831,75 @@
       </c>
       <c r="J34" s="2" t="inlineStr">
         <is>
-          <t>https://admin.shopify.com/store/mccormackpharmacy/products/15671253991755</t>
+          <t>https://admin.shopify.com/store/mccormackpharmacy/products/15671259169099</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="2" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="B35" s="2" t="inlineStr">
         <is>
-          <t>Extra or padded digits</t>
-        </is>
-      </c>
-      <c r="C35" s="2" t="inlineStr">
-        <is>
-          <t>BUNDLE: shop-made, should have no barcode; leave blank</t>
-        </is>
-      </c>
+          <t>No automatic fix</t>
+        </is>
+      </c>
+      <c r="C35" s="2" t="inlineStr"/>
       <c r="D35" s="2" t="inlineStr">
         <is>
-          <t>Unisex Festival Essentials Bundle</t>
+          <t>3 Piece Ladies Set Libertie</t>
         </is>
       </c>
       <c r="E35" s="2" t="inlineStr">
         <is>
-          <t>743485657575858</t>
+          <t>6294015191298</t>
         </is>
       </c>
       <c r="F35" s="2" t="inlineStr"/>
-      <c r="G35" s="2" t="inlineStr">
-        <is>
-          <t>7434856575758</t>
-        </is>
-      </c>
+      <c r="G35" s="2" t="inlineStr"/>
       <c r="H35" s="3" t="inlineStr"/>
       <c r="I35" s="2" t="inlineStr">
         <is>
-          <t>Too many digits; trimming gives a number that passes the check, but 1 in 10 wrong numbers also pass. Check the box.</t>
+          <t>No simple repair. Read the barcode off the box.</t>
         </is>
       </c>
       <c r="J35" s="2" t="inlineStr">
         <is>
-          <t>https://admin.shopify.com/store/mccormackpharmacy/products/15671337877835</t>
+          <t>https://admin.shopify.com/store/mccormackpharmacy/products/15671299834187</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="2" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="B36" s="2" t="inlineStr">
         <is>
-          <t>Extra or padded digits</t>
+          <t>No automatic fix</t>
         </is>
       </c>
       <c r="C36" s="2" t="inlineStr"/>
       <c r="D36" s="2" t="inlineStr">
         <is>
-          <t>Ysl Black Opium Ladies 50Ml Edp Spr</t>
+          <t>Alflorex Precision Biotics-3 Month Supply</t>
         </is>
       </c>
       <c r="E36" s="2" t="inlineStr">
         <is>
-          <t>33654407879190</t>
+          <t>5392000067418</t>
         </is>
       </c>
       <c r="F36" s="2" t="inlineStr"/>
-      <c r="G36" s="2" t="inlineStr">
-        <is>
-          <t>3365440787919</t>
-        </is>
-      </c>
+      <c r="G36" s="2" t="inlineStr"/>
       <c r="H36" s="3" t="inlineStr"/>
       <c r="I36" s="2" t="inlineStr">
         <is>
-          <t>Too many digits; trimming gives a number that passes the check, but 1 in 10 wrong numbers also pass. Check the box.</t>
+          <t>No simple repair. Read the barcode off the box.</t>
         </is>
       </c>
       <c r="J36" s="2" t="inlineStr">
         <is>
-          <t>https://admin.shopify.com/store/mccormackpharmacy/products/15671259169099</t>
+          <t>https://admin.shopify.com/store/mccormackpharmacy/products/15671404659019</t>
         </is>
       </c>
     </row>
@@ -1935,12 +1915,12 @@
       <c r="C37" s="2" t="inlineStr"/>
       <c r="D37" s="2" t="inlineStr">
         <is>
-          <t>3 Piece Ladies Set Libertie</t>
+          <t>Apple Cider Mega Strength 1000Mg Tabs (30 Pk)</t>
         </is>
       </c>
       <c r="E37" s="2" t="inlineStr">
         <is>
-          <t>6294015191298</t>
+          <t>5021827447800</t>
         </is>
       </c>
       <c r="F37" s="2" t="inlineStr"/>
@@ -1953,7 +1933,7 @@
       </c>
       <c r="J37" s="2" t="inlineStr">
         <is>
-          <t>https://admin.shopify.com/store/mccormackpharmacy/products/15671299834187</t>
+          <t>https://admin.shopify.com/store/mccormackpharmacy/products/15671352918347</t>
         </is>
       </c>
     </row>
@@ -1969,12 +1949,12 @@
       <c r="C38" s="2" t="inlineStr"/>
       <c r="D38" s="2" t="inlineStr">
         <is>
-          <t>Alflorex Precision Biotics-3 Month Supply</t>
+          <t>Compeed Discreet Cold Sore</t>
         </is>
       </c>
       <c r="E38" s="2" t="inlineStr">
         <is>
-          <t>5392000067418</t>
+          <t>366355500211</t>
         </is>
       </c>
       <c r="F38" s="2" t="inlineStr"/>
@@ -1987,7 +1967,7 @@
       </c>
       <c r="J38" s="2" t="inlineStr">
         <is>
-          <t>https://admin.shopify.com/store/mccormackpharmacy/products/15671404659019</t>
+          <t>https://admin.shopify.com/store/mccormackpharmacy/products/15671382049099</t>
         </is>
       </c>
     </row>
@@ -2003,12 +1983,12 @@
       <c r="C39" s="2" t="inlineStr"/>
       <c r="D39" s="2" t="inlineStr">
         <is>
-          <t>Apple Cider Mega Strength 1000Mg Tabs (30 Pk)</t>
+          <t>Diesel Only The Brave 50Ml Edt Spr</t>
         </is>
       </c>
       <c r="E39" s="2" t="inlineStr">
         <is>
-          <t>5021827447800</t>
+          <t>0951577468</t>
         </is>
       </c>
       <c r="F39" s="2" t="inlineStr"/>
@@ -2021,7 +2001,7 @@
       </c>
       <c r="J39" s="2" t="inlineStr">
         <is>
-          <t>https://admin.shopify.com/store/mccormackpharmacy/products/15671352918347</t>
+          <t>https://admin.shopify.com/store/mccormackpharmacy/products/15671317823819</t>
         </is>
       </c>
     </row>
@@ -2037,12 +2017,12 @@
       <c r="C40" s="2" t="inlineStr"/>
       <c r="D40" s="2" t="inlineStr">
         <is>
-          <t>Compeed Discreet Cold Sore</t>
+          <t>Estee Lauder Double Wear Makeup Pump</t>
         </is>
       </c>
       <c r="E40" s="2" t="inlineStr">
         <is>
-          <t>366355500211</t>
+          <t>587167188877</t>
         </is>
       </c>
       <c r="F40" s="2" t="inlineStr"/>
@@ -2055,7 +2035,7 @@
       </c>
       <c r="J40" s="2" t="inlineStr">
         <is>
-          <t>https://admin.shopify.com/store/mccormackpharmacy/products/15671382049099</t>
+          <t>https://admin.shopify.com/store/mccormackpharmacy/products/15671270310219</t>
         </is>
       </c>
     </row>
@@ -2071,12 +2051,12 @@
       <c r="C41" s="2" t="inlineStr"/>
       <c r="D41" s="2" t="inlineStr">
         <is>
-          <t>Diesel Only The Brave 50Ml Edt Spr</t>
+          <t>Eylure Brow Dye (Light Brown)</t>
         </is>
       </c>
       <c r="E41" s="2" t="inlineStr">
         <is>
-          <t>0951577468</t>
+          <t>61923200349</t>
         </is>
       </c>
       <c r="F41" s="2" t="inlineStr"/>
@@ -2089,7 +2069,7 @@
       </c>
       <c r="J41" s="2" t="inlineStr">
         <is>
-          <t>https://admin.shopify.com/store/mccormackpharmacy/products/15671317823819</t>
+          <t>https://admin.shopify.com/store/mccormackpharmacy/products/15671325983051</t>
         </is>
       </c>
     </row>
@@ -2102,15 +2082,19 @@
           <t>No automatic fix</t>
         </is>
       </c>
-      <c r="C42" s="2" t="inlineStr"/>
+      <c r="C42" s="2" t="inlineStr">
+        <is>
+          <t>BUNDLE: shop-made, should have no barcode; leave blank</t>
+        </is>
+      </c>
       <c r="D42" s="2" t="inlineStr">
         <is>
-          <t>Estee Lauder Double Wear Makeup Pump</t>
+          <t>Hismile Teeth Whitening &amp; Brightening Bundle</t>
         </is>
       </c>
       <c r="E42" s="2" t="inlineStr">
         <is>
-          <t>587167188877</t>
+          <t>109834869865</t>
         </is>
       </c>
       <c r="F42" s="2" t="inlineStr"/>
@@ -2123,7 +2107,7 @@
       </c>
       <c r="J42" s="2" t="inlineStr">
         <is>
-          <t>https://admin.shopify.com/store/mccormackpharmacy/products/15671270310219</t>
+          <t>https://admin.shopify.com/store/mccormackpharmacy/products/15671374250315</t>
         </is>
       </c>
     </row>
@@ -2139,12 +2123,12 @@
       <c r="C43" s="2" t="inlineStr"/>
       <c r="D43" s="2" t="inlineStr">
         <is>
-          <t>Eylure Brow Dye (Light Brown)</t>
+          <t>Jakemans Cherry Soothing Menthol Lozenges 73G</t>
         </is>
       </c>
       <c r="E43" s="2" t="inlineStr">
         <is>
-          <t>61923200349</t>
+          <t>503104005149</t>
         </is>
       </c>
       <c r="F43" s="2" t="inlineStr"/>
@@ -2157,7 +2141,7 @@
       </c>
       <c r="J43" s="2" t="inlineStr">
         <is>
-          <t>https://admin.shopify.com/store/mccormackpharmacy/products/15671325983051</t>
+          <t>https://admin.shopify.com/store/mccormackpharmacy/products/15671389684043</t>
         </is>
       </c>
     </row>
@@ -2170,19 +2154,15 @@
           <t>No automatic fix</t>
         </is>
       </c>
-      <c r="C44" s="2" t="inlineStr">
-        <is>
-          <t>BUNDLE: shop-made, should have no barcode; leave blank</t>
-        </is>
-      </c>
+      <c r="C44" s="2" t="inlineStr"/>
       <c r="D44" s="2" t="inlineStr">
         <is>
-          <t>Hismile Teeth Whitening &amp; Brightening Bundle</t>
+          <t>King Hair &amp; Beauty Miracle Mist 7 In 1 Spray</t>
         </is>
       </c>
       <c r="E44" s="2" t="inlineStr">
         <is>
-          <t>109834869865</t>
+          <t>4560405959</t>
         </is>
       </c>
       <c r="F44" s="2" t="inlineStr"/>
@@ -2195,7 +2175,7 @@
       </c>
       <c r="J44" s="2" t="inlineStr">
         <is>
-          <t>https://admin.shopify.com/store/mccormackpharmacy/products/15671374250315</t>
+          <t>https://admin.shopify.com/store/mccormackpharmacy/products/15671364813131</t>
         </is>
       </c>
     </row>
@@ -2211,12 +2191,12 @@
       <c r="C45" s="2" t="inlineStr"/>
       <c r="D45" s="2" t="inlineStr">
         <is>
-          <t>Jakemans Cherry Soothing Menthol Lozenges 73G</t>
+          <t>L'il Critters Gummy Vites Multi Vitamin &amp; Mineral Formula 70Pk</t>
         </is>
       </c>
       <c r="E45" s="2" t="inlineStr">
         <is>
-          <t>503104005149</t>
+          <t>2791701757</t>
         </is>
       </c>
       <c r="F45" s="2" t="inlineStr"/>
@@ -2229,7 +2209,7 @@
       </c>
       <c r="J45" s="2" t="inlineStr">
         <is>
-          <t>https://admin.shopify.com/store/mccormackpharmacy/products/15671389684043</t>
+          <t>https://admin.shopify.com/store/mccormackpharmacy/products/15671327785291</t>
         </is>
       </c>
     </row>
@@ -2245,12 +2225,12 @@
       <c r="C46" s="2" t="inlineStr"/>
       <c r="D46" s="2" t="inlineStr">
         <is>
-          <t>King Hair &amp; Beauty Miracle Mist 7 In 1 Spray</t>
+          <t>Luna By Lisa Jordan Lip Balm &amp; Scrub Duo</t>
         </is>
       </c>
       <c r="E46" s="2" t="inlineStr">
         <is>
-          <t>4560405959</t>
+          <t>56789616525</t>
         </is>
       </c>
       <c r="F46" s="2" t="inlineStr"/>
@@ -2263,7 +2243,7 @@
       </c>
       <c r="J46" s="2" t="inlineStr">
         <is>
-          <t>https://admin.shopify.com/store/mccormackpharmacy/products/15671364813131</t>
+          <t>https://admin.shopify.com/store/mccormackpharmacy/products/15671337156939</t>
         </is>
       </c>
     </row>
@@ -2279,12 +2259,12 @@
       <c r="C47" s="2" t="inlineStr"/>
       <c r="D47" s="2" t="inlineStr">
         <is>
-          <t>L'il Critters Gummy Vites Multi Vitamin &amp; Mineral Formula 70Pk</t>
+          <t>Mam Colours Of Nature 0+ Months (Blue/White Fox)</t>
         </is>
       </c>
       <c r="E47" s="2" t="inlineStr">
         <is>
-          <t>2791701757</t>
+          <t>900161681380000</t>
         </is>
       </c>
       <c r="F47" s="2" t="inlineStr"/>
@@ -2297,7 +2277,7 @@
       </c>
       <c r="J47" s="2" t="inlineStr">
         <is>
-          <t>https://admin.shopify.com/store/mccormackpharmacy/products/15671327785291</t>
+          <t>https://admin.shopify.com/store/mccormackpharmacy/products/15671363699019</t>
         </is>
       </c>
     </row>
@@ -2313,12 +2293,12 @@
       <c r="C48" s="2" t="inlineStr"/>
       <c r="D48" s="2" t="inlineStr">
         <is>
-          <t>Luna By Lisa Jordan Lip Balm &amp; Scrub Duo</t>
+          <t>Mam Easy Start Anti-Colic 0+Months</t>
         </is>
       </c>
       <c r="E48" s="2" t="inlineStr">
         <is>
-          <t>56789616525</t>
+          <t>901616620058</t>
         </is>
       </c>
       <c r="F48" s="2" t="inlineStr"/>
@@ -2331,7 +2311,7 @@
       </c>
       <c r="J48" s="2" t="inlineStr">
         <is>
-          <t>https://admin.shopify.com/store/mccormackpharmacy/products/15671337156939</t>
+          <t>https://admin.shopify.com/store/mccormackpharmacy/products/15671339680075</t>
         </is>
       </c>
     </row>
@@ -2347,12 +2327,12 @@
       <c r="C49" s="2" t="inlineStr"/>
       <c r="D49" s="2" t="inlineStr">
         <is>
-          <t>Mam Colours Of Nature 0+ Months (Blue/White Fox)</t>
+          <t>Nivea Men Clean Shave Kit</t>
         </is>
       </c>
       <c r="E49" s="2" t="inlineStr">
         <is>
-          <t>900161681380000</t>
+          <t>025970012858</t>
         </is>
       </c>
       <c r="F49" s="2" t="inlineStr"/>
@@ -2365,7 +2345,7 @@
       </c>
       <c r="J49" s="2" t="inlineStr">
         <is>
-          <t>https://admin.shopify.com/store/mccormackpharmacy/products/15671363699019</t>
+          <t>https://admin.shopify.com/store/mccormackpharmacy/products/15671356916043</t>
         </is>
       </c>
     </row>
@@ -2381,12 +2361,12 @@
       <c r="C50" s="2" t="inlineStr"/>
       <c r="D50" s="2" t="inlineStr">
         <is>
-          <t>Mam Easy Start Anti-Colic 0+Months</t>
+          <t>Nivea Men Feeling Protected Gift Set</t>
         </is>
       </c>
       <c r="E50" s="2" t="inlineStr">
         <is>
-          <t>901616620058</t>
+          <t>025970014791</t>
         </is>
       </c>
       <c r="F50" s="2" t="inlineStr"/>
@@ -2399,7 +2379,7 @@
       </c>
       <c r="J50" s="2" t="inlineStr">
         <is>
-          <t>https://admin.shopify.com/store/mccormackpharmacy/products/15671339680075</t>
+          <t>https://admin.shopify.com/store/mccormackpharmacy/products/15671375331659</t>
         </is>
       </c>
     </row>
@@ -2415,12 +2395,12 @@
       <c r="C51" s="2" t="inlineStr"/>
       <c r="D51" s="2" t="inlineStr">
         <is>
-          <t>Nivea Men Clean Shave Kit</t>
+          <t>Nuage Hayfever Barrier Balm 50G</t>
         </is>
       </c>
       <c r="E51" s="2" t="inlineStr">
         <is>
-          <t>025970012858</t>
+          <t>6278390031</t>
         </is>
       </c>
       <c r="F51" s="2" t="inlineStr"/>
@@ -2433,7 +2413,7 @@
       </c>
       <c r="J51" s="2" t="inlineStr">
         <is>
-          <t>https://admin.shopify.com/store/mccormackpharmacy/products/15671356916043</t>
+          <t>https://admin.shopify.com/store/mccormackpharmacy/products/15671390339403</t>
         </is>
       </c>
     </row>
@@ -2449,12 +2429,12 @@
       <c r="C52" s="2" t="inlineStr"/>
       <c r="D52" s="2" t="inlineStr">
         <is>
-          <t>Nivea Men Feeling Protected Gift Set</t>
+          <t>Nuage Hayfever Relief Wipes 30Pk</t>
         </is>
       </c>
       <c r="E52" s="2" t="inlineStr">
         <is>
-          <t>025970014791</t>
+          <t>26789030980</t>
         </is>
       </c>
       <c r="F52" s="2" t="inlineStr"/>
@@ -2467,7 +2447,7 @@
       </c>
       <c r="J52" s="2" t="inlineStr">
         <is>
-          <t>https://admin.shopify.com/store/mccormackpharmacy/products/15671375331659</t>
+          <t>https://admin.shopify.com/store/mccormackpharmacy/products/15671289086283</t>
         </is>
       </c>
     </row>
@@ -2483,12 +2463,12 @@
       <c r="C53" s="2" t="inlineStr"/>
       <c r="D53" s="2" t="inlineStr">
         <is>
-          <t>Nuage Hayfever Barrier Balm 50G</t>
+          <t>Optibac Babies &amp; Children 0-12 Years (30 Sachets)</t>
         </is>
       </c>
       <c r="E53" s="2" t="inlineStr">
         <is>
-          <t>6278390031</t>
+          <t>506008661028</t>
         </is>
       </c>
       <c r="F53" s="2" t="inlineStr"/>
@@ -2501,7 +2481,7 @@
       </c>
       <c r="J53" s="2" t="inlineStr">
         <is>
-          <t>https://admin.shopify.com/store/mccormackpharmacy/products/15671390339403</t>
+          <t>https://admin.shopify.com/store/mccormackpharmacy/products/15671319363915</t>
         </is>
       </c>
     </row>
@@ -2514,15 +2494,19 @@
           <t>No automatic fix</t>
         </is>
       </c>
-      <c r="C54" s="2" t="inlineStr"/>
+      <c r="C54" s="2" t="inlineStr">
+        <is>
+          <t>BUNDLE: shop-made, should have no barcode; leave blank</t>
+        </is>
+      </c>
       <c r="D54" s="2" t="inlineStr">
         <is>
-          <t>Nuage Hayfever Relief Wipes 30Pk</t>
+          <t>Pestle &amp; Mortar Essentials Body Wash &amp; Body Cream 500Ml Bundle</t>
         </is>
       </c>
       <c r="E54" s="2" t="inlineStr">
         <is>
-          <t>26789030980</t>
+          <t>0000000</t>
         </is>
       </c>
       <c r="F54" s="2" t="inlineStr"/>
@@ -2535,7 +2519,7 @@
       </c>
       <c r="J54" s="2" t="inlineStr">
         <is>
-          <t>https://admin.shopify.com/store/mccormackpharmacy/products/15671289086283</t>
+          <t>https://admin.shopify.com/store/mccormackpharmacy/products/15671379231051</t>
         </is>
       </c>
     </row>
@@ -2548,15 +2532,19 @@
           <t>No automatic fix</t>
         </is>
       </c>
-      <c r="C55" s="2" t="inlineStr"/>
+      <c r="C55" s="2" t="inlineStr">
+        <is>
+          <t>BUNDLE: shop-made, should have no barcode; leave blank</t>
+        </is>
+      </c>
       <c r="D55" s="2" t="inlineStr">
         <is>
-          <t>Optibac Babies &amp; Children 0-12 Years (30 Sachets)</t>
+          <t>Pestle &amp; Mortar Essentials Bundle</t>
         </is>
       </c>
       <c r="E55" s="2" t="inlineStr">
         <is>
-          <t>506008661028</t>
+          <t>038548748843</t>
         </is>
       </c>
       <c r="F55" s="2" t="inlineStr"/>
@@ -2569,7 +2557,7 @@
       </c>
       <c r="J55" s="2" t="inlineStr">
         <is>
-          <t>https://admin.shopify.com/store/mccormackpharmacy/products/15671319363915</t>
+          <t>https://admin.shopify.com/store/mccormackpharmacy/products/15671357079883</t>
         </is>
       </c>
     </row>
@@ -2589,12 +2577,12 @@
       </c>
       <c r="D56" s="2" t="inlineStr">
         <is>
-          <t>Pestle &amp; Mortar Essentials Body Wash &amp; Body Cream 500Ml Bundle</t>
+          <t>Pestle &amp; Mortar Hand Wash &amp; Hand Cream Bundle</t>
         </is>
       </c>
       <c r="E56" s="2" t="inlineStr">
         <is>
-          <t>0000000</t>
+          <t>111111</t>
         </is>
       </c>
       <c r="F56" s="2" t="inlineStr"/>
@@ -2607,7 +2595,7 @@
       </c>
       <c r="J56" s="2" t="inlineStr">
         <is>
-          <t>https://admin.shopify.com/store/mccormackpharmacy/products/15671379231051</t>
+          <t>https://admin.shopify.com/store/mccormackpharmacy/products/15671342006603</t>
         </is>
       </c>
     </row>
@@ -2627,12 +2615,12 @@
       </c>
       <c r="D57" s="2" t="inlineStr">
         <is>
-          <t>Pestle &amp; Mortar Essentials Bundle</t>
+          <t>Pestle &amp; Mortar Hydrate And Vit C Bundle</t>
         </is>
       </c>
       <c r="E57" s="2" t="inlineStr">
         <is>
-          <t>038548748843</t>
+          <t>11111</t>
         </is>
       </c>
       <c r="F57" s="2" t="inlineStr"/>
@@ -2645,7 +2633,7 @@
       </c>
       <c r="J57" s="2" t="inlineStr">
         <is>
-          <t>https://admin.shopify.com/store/mccormackpharmacy/products/15671357079883</t>
+          <t>https://admin.shopify.com/store/mccormackpharmacy/products/15671277519179</t>
         </is>
       </c>
     </row>
@@ -2665,12 +2653,12 @@
       </c>
       <c r="D58" s="2" t="inlineStr">
         <is>
-          <t>Pestle &amp; Mortar Hand Wash &amp; Hand Cream Bundle</t>
+          <t>Pestle &amp; Mortar Hydration Bundle</t>
         </is>
       </c>
       <c r="E58" s="2" t="inlineStr">
         <is>
-          <t>111111</t>
+          <t>75748438398</t>
         </is>
       </c>
       <c r="F58" s="2" t="inlineStr"/>
@@ -2683,7 +2671,7 @@
       </c>
       <c r="J58" s="2" t="inlineStr">
         <is>
-          <t>https://admin.shopify.com/store/mccormackpharmacy/products/15671342006603</t>
+          <t>https://admin.shopify.com/store/mccormackpharmacy/products/15671297573195</t>
         </is>
       </c>
     </row>
@@ -2696,19 +2684,15 @@
           <t>No automatic fix</t>
         </is>
       </c>
-      <c r="C59" s="2" t="inlineStr">
-        <is>
-          <t>BUNDLE: shop-made, should have no barcode; leave blank</t>
-        </is>
-      </c>
+      <c r="C59" s="2" t="inlineStr"/>
       <c r="D59" s="2" t="inlineStr">
         <is>
-          <t>Pestle &amp; Mortar Hydrate And Vit C Bundle</t>
+          <t>Red Door 100Ml Edt</t>
         </is>
       </c>
       <c r="E59" s="2" t="inlineStr">
         <is>
-          <t>11111</t>
+          <t>805805558420</t>
         </is>
       </c>
       <c r="F59" s="2" t="inlineStr"/>
@@ -2721,7 +2705,7 @@
       </c>
       <c r="J59" s="2" t="inlineStr">
         <is>
-          <t>https://admin.shopify.com/store/mccormackpharmacy/products/15671277519179</t>
+          <t>https://admin.shopify.com/store/mccormackpharmacy/products/15671413080395</t>
         </is>
       </c>
     </row>
@@ -2734,19 +2718,15 @@
           <t>No automatic fix</t>
         </is>
       </c>
-      <c r="C60" s="2" t="inlineStr">
-        <is>
-          <t>BUNDLE: shop-made, should have no barcode; leave blank</t>
-        </is>
-      </c>
+      <c r="C60" s="2" t="inlineStr"/>
       <c r="D60" s="2" t="inlineStr">
         <is>
-          <t>Pestle &amp; Mortar Hydration Bundle</t>
+          <t>Revive Active 3 Month Supply - 90 Sachets</t>
         </is>
       </c>
       <c r="E60" s="2" t="inlineStr">
         <is>
-          <t>75748438398</t>
+          <t>5391517512176</t>
         </is>
       </c>
       <c r="F60" s="2" t="inlineStr"/>
@@ -2759,7 +2739,7 @@
       </c>
       <c r="J60" s="2" t="inlineStr">
         <is>
-          <t>https://admin.shopify.com/store/mccormackpharmacy/products/15671297573195</t>
+          <t>https://admin.shopify.com/store/mccormackpharmacy/products/15671372054859</t>
         </is>
       </c>
     </row>
@@ -2775,12 +2755,12 @@
       <c r="C61" s="2" t="inlineStr"/>
       <c r="D61" s="2" t="inlineStr">
         <is>
-          <t>Red Door 100Ml Edt</t>
+          <t>Revive Active 6 Month Supply -180 Sachets</t>
         </is>
       </c>
       <c r="E61" s="2" t="inlineStr">
         <is>
-          <t>805805558420</t>
+          <t>5391517512177</t>
         </is>
       </c>
       <c r="F61" s="2" t="inlineStr"/>
@@ -2793,7 +2773,7 @@
       </c>
       <c r="J61" s="2" t="inlineStr">
         <is>
-          <t>https://admin.shopify.com/store/mccormackpharmacy/products/15671413080395</t>
+          <t>https://admin.shopify.com/store/mccormackpharmacy/products/15671333585227</t>
         </is>
       </c>
     </row>
@@ -2809,12 +2789,12 @@
       <c r="C62" s="2" t="inlineStr"/>
       <c r="D62" s="2" t="inlineStr">
         <is>
-          <t>Revive Active 3 Month Supply - 90 Sachets</t>
+          <t>Revive Active Zest- 3 Month Supply-90 Sachets</t>
         </is>
       </c>
       <c r="E62" s="2" t="inlineStr">
         <is>
-          <t>5391517512176</t>
+          <t>735850866841</t>
         </is>
       </c>
       <c r="F62" s="2" t="inlineStr"/>
@@ -2827,7 +2807,7 @@
       </c>
       <c r="J62" s="2" t="inlineStr">
         <is>
-          <t>https://admin.shopify.com/store/mccormackpharmacy/products/15671372054859</t>
+          <t>https://admin.shopify.com/store/mccormackpharmacy/products/15671370187083</t>
         </is>
       </c>
     </row>
@@ -2843,12 +2823,12 @@
       <c r="C63" s="2" t="inlineStr"/>
       <c r="D63" s="2" t="inlineStr">
         <is>
-          <t>Revive Active 6 Month Supply -180 Sachets</t>
+          <t>Revive Tropical 3 Month Supply - 90 Sachets</t>
         </is>
       </c>
       <c r="E63" s="2" t="inlineStr">
         <is>
-          <t>5391517512177</t>
+          <t>079775747684</t>
         </is>
       </c>
       <c r="F63" s="2" t="inlineStr"/>
@@ -2861,7 +2841,7 @@
       </c>
       <c r="J63" s="2" t="inlineStr">
         <is>
-          <t>https://admin.shopify.com/store/mccormackpharmacy/products/15671333585227</t>
+          <t>https://admin.shopify.com/store/mccormackpharmacy/products/15671388471627</t>
         </is>
       </c>
     </row>
@@ -2877,12 +2857,12 @@
       <c r="C64" s="2" t="inlineStr"/>
       <c r="D64" s="2" t="inlineStr">
         <is>
-          <t>Revive Active Zest- 3 Month Supply-90 Sachets</t>
+          <t>Sculpted Velvet Veil Invisible Loose Setting Powder</t>
         </is>
       </c>
       <c r="E64" s="2" t="inlineStr">
         <is>
-          <t>735850866841</t>
+          <t>794712490866</t>
         </is>
       </c>
       <c r="F64" s="2" t="inlineStr"/>
@@ -2895,7 +2875,7 @@
       </c>
       <c r="J64" s="2" t="inlineStr">
         <is>
-          <t>https://admin.shopify.com/store/mccormackpharmacy/products/15671370187083</t>
+          <t>https://admin.shopify.com/store/mccormackpharmacy/products/15671410065739</t>
         </is>
       </c>
     </row>
@@ -2911,12 +2891,12 @@
       <c r="C65" s="2" t="inlineStr"/>
       <c r="D65" s="2" t="inlineStr">
         <is>
-          <t>Revive Tropical 3 Month Supply - 90 Sachets</t>
+          <t>Tena Pants Plus (Extra Large)</t>
         </is>
       </c>
       <c r="E65" s="2" t="inlineStr">
         <is>
-          <t>079775747684</t>
+          <t>13232120</t>
         </is>
       </c>
       <c r="F65" s="2" t="inlineStr"/>
@@ -2929,7 +2909,7 @@
       </c>
       <c r="J65" s="2" t="inlineStr">
         <is>
-          <t>https://admin.shopify.com/store/mccormackpharmacy/products/15671388471627</t>
+          <t>https://admin.shopify.com/store/mccormackpharmacy/products/15671403446603</t>
         </is>
       </c>
     </row>
@@ -2945,12 +2925,12 @@
       <c r="C66" s="2" t="inlineStr"/>
       <c r="D66" s="2" t="inlineStr">
         <is>
-          <t>Sculpted Velvet Veil Invisible Loose Setting Powder</t>
+          <t>Travel Blue Comfort Bands</t>
         </is>
       </c>
       <c r="E66" s="2" t="inlineStr">
         <is>
-          <t>794712490866</t>
+          <t>501840400501</t>
         </is>
       </c>
       <c r="F66" s="2" t="inlineStr"/>
@@ -2963,7 +2943,7 @@
       </c>
       <c r="J66" s="2" t="inlineStr">
         <is>
-          <t>https://admin.shopify.com/store/mccormackpharmacy/products/15671410065739</t>
+          <t>https://admin.shopify.com/store/mccormackpharmacy/products/15671302062411</t>
         </is>
       </c>
     </row>
@@ -2979,12 +2959,12 @@
       <c r="C67" s="2" t="inlineStr"/>
       <c r="D67" s="2" t="inlineStr">
         <is>
-          <t>Tena Pants Plus (Extra Large)</t>
+          <t>Voduz Clear It Exfoliating Scalp Scrub</t>
         </is>
       </c>
       <c r="E67" s="2" t="inlineStr">
         <is>
-          <t>13232120</t>
+          <t>5060806565008</t>
         </is>
       </c>
       <c r="F67" s="2" t="inlineStr"/>
@@ -2997,7 +2977,7 @@
       </c>
       <c r="J67" s="2" t="inlineStr">
         <is>
-          <t>https://admin.shopify.com/store/mccormackpharmacy/products/15671403446603</t>
+          <t>https://admin.shopify.com/store/mccormackpharmacy/products/15671391289675</t>
         </is>
       </c>
     </row>
@@ -3013,12 +2993,12 @@
       <c r="C68" s="2" t="inlineStr"/>
       <c r="D68" s="2" t="inlineStr">
         <is>
-          <t>Travel Blue Comfort Bands</t>
+          <t>Voduz Sun Soothe After Sun Leave In Fluid 90Ml</t>
         </is>
       </c>
       <c r="E68" s="2" t="inlineStr">
         <is>
-          <t>501840400501</t>
+          <t>5060939587221</t>
         </is>
       </c>
       <c r="F68" s="2" t="inlineStr"/>
@@ -3031,7 +3011,7 @@
       </c>
       <c r="J68" s="2" t="inlineStr">
         <is>
-          <t>https://admin.shopify.com/store/mccormackpharmacy/products/15671302062411</t>
+          <t>https://admin.shopify.com/store/mccormackpharmacy/products/15671282336075</t>
         </is>
       </c>
     </row>
@@ -3047,12 +3027,12 @@
       <c r="C69" s="2" t="inlineStr"/>
       <c r="D69" s="2" t="inlineStr">
         <is>
-          <t>Voduz Clear It Exfoliating Scalp Scrub</t>
+          <t>Voduz Velvet Crown 200Ml</t>
         </is>
       </c>
       <c r="E69" s="2" t="inlineStr">
         <is>
-          <t>5060806565008</t>
+          <t>079359168304</t>
         </is>
       </c>
       <c r="F69" s="2" t="inlineStr"/>
@@ -3065,7 +3045,7 @@
       </c>
       <c r="J69" s="2" t="inlineStr">
         <is>
-          <t>https://admin.shopify.com/store/mccormackpharmacy/products/15671391289675</t>
+          <t>https://admin.shopify.com/store/mccormackpharmacy/products/15671307829579</t>
         </is>
       </c>
     </row>
@@ -3081,12 +3061,12 @@
       <c r="C70" s="2" t="inlineStr"/>
       <c r="D70" s="2" t="inlineStr">
         <is>
-          <t>Voduz Sun Soothe After Sun Leave In Fluid 90Ml</t>
+          <t>Water Wipes- 24 Pack</t>
         </is>
       </c>
       <c r="E70" s="2" t="inlineStr">
         <is>
-          <t>5060939587221</t>
+          <t>35614643163</t>
         </is>
       </c>
       <c r="F70" s="2" t="inlineStr"/>
@@ -3099,7 +3079,7 @@
       </c>
       <c r="J70" s="2" t="inlineStr">
         <is>
-          <t>https://admin.shopify.com/store/mccormackpharmacy/products/15671282336075</t>
+          <t>https://admin.shopify.com/store/mccormackpharmacy/products/15671280501067</t>
         </is>
       </c>
     </row>
@@ -3115,12 +3095,12 @@
       <c r="C71" s="2" t="inlineStr"/>
       <c r="D71" s="2" t="inlineStr">
         <is>
-          <t>Voduz Velvet Crown 200Ml</t>
+          <t>Waxperts Beautiful Body Oil</t>
         </is>
       </c>
       <c r="E71" s="2" t="inlineStr">
         <is>
-          <t>079359168304</t>
+          <t>21542515912</t>
         </is>
       </c>
       <c r="F71" s="2" t="inlineStr"/>
@@ -3133,7 +3113,7 @@
       </c>
       <c r="J71" s="2" t="inlineStr">
         <is>
-          <t>https://admin.shopify.com/store/mccormackpharmacy/products/15671307829579</t>
+          <t>https://admin.shopify.com/store/mccormackpharmacy/products/15671338500427</t>
         </is>
       </c>
     </row>
@@ -3149,12 +3129,12 @@
       <c r="C72" s="2" t="inlineStr"/>
       <c r="D72" s="2" t="inlineStr">
         <is>
-          <t>Water Wipes- 24 Pack</t>
+          <t>Wild Fresh Cotton &amp; Sea Salt Mens Refill</t>
         </is>
       </c>
       <c r="E72" s="2" t="inlineStr">
         <is>
-          <t>35614643163</t>
+          <t>506500399070</t>
         </is>
       </c>
       <c r="F72" s="2" t="inlineStr"/>
@@ -3167,7 +3147,7 @@
       </c>
       <c r="J72" s="2" t="inlineStr">
         <is>
-          <t>https://admin.shopify.com/store/mccormackpharmacy/products/15671280501067</t>
+          <t>https://admin.shopify.com/store/mccormackpharmacy/products/15671320019275</t>
         </is>
       </c>
     </row>
@@ -3183,12 +3163,12 @@
       <c r="C73" s="2" t="inlineStr"/>
       <c r="D73" s="2" t="inlineStr">
         <is>
-          <t>Waxperts Beautiful Body Oil</t>
+          <t>Wild Green Case Mint &amp; Aloe Vera Mens Starter Pack</t>
         </is>
       </c>
       <c r="E73" s="2" t="inlineStr">
         <is>
-          <t>21542515912</t>
+          <t>50650003990685</t>
         </is>
       </c>
       <c r="F73" s="2" t="inlineStr"/>
@@ -3201,80 +3181,12 @@
       </c>
       <c r="J73" s="2" t="inlineStr">
         <is>
-          <t>https://admin.shopify.com/store/mccormackpharmacy/products/15671338500427</t>
-        </is>
-      </c>
-    </row>
-    <row r="74">
-      <c r="A74" s="2" t="n">
-        <v>5</v>
-      </c>
-      <c r="B74" s="2" t="inlineStr">
-        <is>
-          <t>No automatic fix</t>
-        </is>
-      </c>
-      <c r="C74" s="2" t="inlineStr"/>
-      <c r="D74" s="2" t="inlineStr">
-        <is>
-          <t>Wild Fresh Cotton &amp; Sea Salt Mens Refill</t>
-        </is>
-      </c>
-      <c r="E74" s="2" t="inlineStr">
-        <is>
-          <t>506500399070</t>
-        </is>
-      </c>
-      <c r="F74" s="2" t="inlineStr"/>
-      <c r="G74" s="2" t="inlineStr"/>
-      <c r="H74" s="3" t="inlineStr"/>
-      <c r="I74" s="2" t="inlineStr">
-        <is>
-          <t>No simple repair. Read the barcode off the box.</t>
-        </is>
-      </c>
-      <c r="J74" s="2" t="inlineStr">
-        <is>
-          <t>https://admin.shopify.com/store/mccormackpharmacy/products/15671320019275</t>
-        </is>
-      </c>
-    </row>
-    <row r="75">
-      <c r="A75" s="2" t="n">
-        <v>5</v>
-      </c>
-      <c r="B75" s="2" t="inlineStr">
-        <is>
-          <t>No automatic fix</t>
-        </is>
-      </c>
-      <c r="C75" s="2" t="inlineStr"/>
-      <c r="D75" s="2" t="inlineStr">
-        <is>
-          <t>Wild Green Case Mint &amp; Aloe Vera Mens Starter Pack</t>
-        </is>
-      </c>
-      <c r="E75" s="2" t="inlineStr">
-        <is>
-          <t>50650003990685</t>
-        </is>
-      </c>
-      <c r="F75" s="2" t="inlineStr"/>
-      <c r="G75" s="2" t="inlineStr"/>
-      <c r="H75" s="3" t="inlineStr"/>
-      <c r="I75" s="2" t="inlineStr">
-        <is>
-          <t>No simple repair. Read the barcode off the box.</t>
-        </is>
-      </c>
-      <c r="J75" s="2" t="inlineStr">
-        <is>
           <t>https://admin.shopify.com/store/mccormackpharmacy/products/15671328342347</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:J75"/>
+  <autoFilter ref="A1:J73"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>